<commit_message>
known group comparison - adding comparison estimates
</commit_message>
<xml_diff>
--- a/estudos/avaliacao_dados/C. Validade externa/C2. Known-group/Comparativo.xlsx
+++ b/estudos/avaliacao_dados/C. Validade externa/C2. Known-group/Comparativo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4fed8d7a7efb8cd6/Trampos/Cebrap/Afro/Projetos/Territorio Negro/analysis/territorios_negros/estudos/avaliacao_dados/C. Validade externa/C2. Known-group/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="87" documentId="8_{4B746B58-273E-4BA3-9203-0EB3E7216C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{914DFB8F-F030-4E1F-A71F-EE37ED9CC392}"/>
+  <xr:revisionPtr revIDLastSave="88" documentId="8_{4B746B58-273E-4BA3-9203-0EB3E7216C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF221024-3201-4EFE-B604-EC3043B06153}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{FB758A09-3C3B-4901-8572-23A69892CF1B}"/>
   </bookViews>
@@ -156,7 +156,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -196,7 +196,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -542,7 +542,7 @@
     <col min="6" max="6" width="9.85546875" customWidth="1"/>
     <col min="7" max="7" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="42.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.140625" customWidth="1"/>
+    <col min="9" max="9" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="33.5703125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="21.42578125" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
known groups - changing column title
</commit_message>
<xml_diff>
--- a/estudos/avaliacao_dados/C. Validade externa/C2. Known-group/Comparativo.xlsx
+++ b/estudos/avaliacao_dados/C. Validade externa/C2. Known-group/Comparativo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4fed8d7a7efb8cd6/Trampos/Cebrap/Afro/Projetos/Territorio Negro/analysis/territorios_negros/estudos/avaliacao_dados/C. Validade externa/C2. Known-group/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="88" documentId="8_{4B746B58-273E-4BA3-9203-0EB3E7216C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF221024-3201-4EFE-B604-EC3043B06153}"/>
+  <xr:revisionPtr revIDLastSave="90" documentId="8_{4B746B58-273E-4BA3-9203-0EB3E7216C76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5F044BE-A368-458F-9C69-BDB5C21DC64A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{FB758A09-3C3B-4901-8572-23A69892CF1B}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="35">
   <si>
     <t>RM</t>
   </si>
@@ -1078,7 +1078,8 @@
     <col min="2" max="2" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="9.85546875" customWidth="1"/>
+    <col min="6" max="6" width="9.85546875" customWidth="1"/>
+    <col min="7" max="7" width="11.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="33.5703125" bestFit="1" customWidth="1"/>
@@ -1101,6 +1102,9 @@
       <c r="F2" t="s">
         <v>4</v>
       </c>
+      <c r="G2" t="s">
+        <v>34</v>
+      </c>
       <c r="H2" t="s">
         <v>10</v>
       </c>

</xml_diff>